<commit_message>
Add contacts sheet to task tracker
Co-authored-by: DenisBerezovski1 <DenisBerezovski1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/office_task_tracker.xlsx
+++ b/office_task_tracker.xlsx
@@ -7,7 +7,8 @@
   <sheets>
     <sheet name="Задачи" sheetId="1" r:id="rId1"/>
     <sheet name="Сводка" sheetId="2" r:id="rId2"/>
-    <sheet name="Настройки" sheetId="3" r:id="rId3"/>
+    <sheet name="Контакты" sheetId="3" r:id="rId3"/>
+    <sheet name="Настройки" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="task_categories">'Настройки'!$A$3:$A$8</definedName>
@@ -4286,6 +4287,654 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FF70AD47"/>
+  </sheetPr>
+  <dimension ref="A1:C122"/>
+  <sheetFormatPr defaultRowHeight="20"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Контакты для рабочих взаимодействий</t>
+        </is>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+    </row>
+    <row r="2" spans="1:3" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ФИО</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Номер телефона</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Почтовый адрес</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="2"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="2"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="2"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="2"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="2"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="2"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="2"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="2"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="2"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="2"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="2"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="2"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="2"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="2"/>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="2"/>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="2"/>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="2"/>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="2"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="2"/>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="2"/>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="2"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="2"/>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="2"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="2"/>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="2"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="2"/>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="2"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="2"/>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="2"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="2"/>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="2"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="2"/>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="2"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="2"/>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="2"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="2"/>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="2"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="2"/>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="2"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="2"/>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="2"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="2"/>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="2"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="2"/>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="2"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="2"/>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="2"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="2"/>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="2"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="2"/>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="2"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="2"/>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="2"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="2"/>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="2"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="2"/>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="2"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="2"/>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="2"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="2"/>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="2"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="2"/>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="2"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="2"/>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="2"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="2"/>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="2"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="2"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="2"/>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="2"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="2"/>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="2"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="2"/>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="2"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="2"/>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="2"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="2"/>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="2"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="2"/>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="2"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="2"/>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="2"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="2"/>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" s="2"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="2"/>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" s="2"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="2"/>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="2"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="2"/>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" s="2"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="2"/>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="2"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="2"/>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="2"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="2"/>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" s="2"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="2"/>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="2"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="2"/>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="2"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="2"/>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="2"/>
+      <c r="B86" s="4"/>
+      <c r="C86" s="2"/>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" s="2"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="2"/>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" s="2"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="2"/>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" s="2"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="2"/>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" s="2"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="2"/>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" s="2"/>
+      <c r="B91" s="4"/>
+      <c r="C91" s="2"/>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" s="2"/>
+      <c r="B92" s="4"/>
+      <c r="C92" s="2"/>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" s="2"/>
+      <c r="B93" s="4"/>
+      <c r="C93" s="2"/>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="2"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="2"/>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="2"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="2"/>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" s="2"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="2"/>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="2"/>
+      <c r="B97" s="4"/>
+      <c r="C97" s="2"/>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="2"/>
+      <c r="B98" s="4"/>
+      <c r="C98" s="2"/>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="2"/>
+      <c r="B99" s="4"/>
+      <c r="C99" s="2"/>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="2"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="2"/>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" s="2"/>
+      <c r="B101" s="4"/>
+      <c r="C101" s="2"/>
+    </row>
+    <row r="102" spans="1:3">
+      <c r="A102" s="2"/>
+      <c r="B102" s="4"/>
+      <c r="C102" s="2"/>
+    </row>
+    <row r="103" spans="1:3">
+      <c r="A103" s="2"/>
+      <c r="B103" s="4"/>
+      <c r="C103" s="2"/>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="A104" s="2"/>
+      <c r="B104" s="4"/>
+      <c r="C104" s="2"/>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" s="2"/>
+      <c r="B105" s="4"/>
+      <c r="C105" s="2"/>
+    </row>
+    <row r="106" spans="1:3">
+      <c r="A106" s="2"/>
+      <c r="B106" s="4"/>
+      <c r="C106" s="2"/>
+    </row>
+    <row r="107" spans="1:3">
+      <c r="A107" s="2"/>
+      <c r="B107" s="4"/>
+      <c r="C107" s="2"/>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" s="2"/>
+      <c r="B108" s="4"/>
+      <c r="C108" s="2"/>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" s="2"/>
+      <c r="B109" s="4"/>
+      <c r="C109" s="2"/>
+    </row>
+    <row r="110" spans="1:3">
+      <c r="A110" s="2"/>
+      <c r="B110" s="4"/>
+      <c r="C110" s="2"/>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" s="2"/>
+      <c r="B111" s="4"/>
+      <c r="C111" s="2"/>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" s="2"/>
+      <c r="B112" s="4"/>
+      <c r="C112" s="2"/>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" s="2"/>
+      <c r="B113" s="4"/>
+      <c r="C113" s="2"/>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="2"/>
+      <c r="B114" s="4"/>
+      <c r="C114" s="2"/>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="2"/>
+      <c r="B115" s="4"/>
+      <c r="C115" s="2"/>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="2"/>
+      <c r="B116" s="4"/>
+      <c r="C116" s="2"/>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="2"/>
+      <c r="B117" s="4"/>
+      <c r="C117" s="2"/>
+    </row>
+    <row r="118" spans="1:3">
+      <c r="A118" s="2"/>
+      <c r="B118" s="4"/>
+      <c r="C118" s="2"/>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" s="2"/>
+      <c r="B119" s="4"/>
+      <c r="C119" s="2"/>
+    </row>
+    <row r="120" spans="1:3">
+      <c r="A120" s="2"/>
+      <c r="B120" s="4"/>
+      <c r="C120" s="2"/>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" s="2"/>
+      <c r="B121" s="4"/>
+      <c r="C121" s="2"/>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" s="2"/>
+      <c r="B122" s="4"/>
+      <c r="C122" s="2"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:C122"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF7F7F7F"/>
   </sheetPr>
   <dimension ref="A1:D8"/>

</xml_diff>

<commit_message>
Link responsible field to contacts
Co-authored-by: DenisBerezovski1 <DenisBerezovski1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/office_task_tracker.xlsx
+++ b/office_task_tracker.xlsx
@@ -14,7 +14,7 @@
     <definedName name="task_categories">'Настройки'!$A$3:$A$8</definedName>
     <definedName name="task_priorities">'Настройки'!$B$3:$B$5</definedName>
     <definedName name="task_statuses">'Настройки'!$C$3:$C$6</definedName>
-    <definedName name="task_employees">'Настройки'!$D$3:$D$7</definedName>
+    <definedName name="contact_names">'Контакты'!$A$4:INDEX('Контакты'!$A:$A,IFERROR(LOOKUP(2,1/(NOT(ISBLANK('Контакты'!$A$4:$A$1048576))),ROW('Контакты'!$A$4:$A$1048576)),4))</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -4122,7 +4122,7 @@
       <formula1>task_categories</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E202">
-      <formula1>task_employees</formula1>
+      <formula1>contact_names</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F202">
       <formula1>task_priorities</formula1>
@@ -4158,7 +4158,7 @@
     <row r="2" spans="1:2" ht="24" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Лист помогает контролировать личные задачи: ответственных можно указывать в основной таблице, но работа ведется из одной вкладки.</t>
+          <t>Лист помогает контролировать личные задачи: ответственных выбирайте из вкладки «Контакты», а работать можно из одной основной таблицы.</t>
         </is>
       </c>
       <c r="B2" s="6"/>
@@ -4289,12 +4289,12 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1" style="2"/>
+    <col min="2" max="2" width="20" customWidth="1" style="4"/>
+    <col min="3" max="3" width="42" customWidth="1" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
@@ -4306,27 +4306,31 @@
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
     </row>
-    <row r="2" spans="1:3" ht="22" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Добавляйте новые строки ниже: список для поля «Ответственный» обновляется автоматически.</t>
+        </is>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" spans="1:3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>ФИО</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Номер телефона</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Почтовый адрес</t>
         </is>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2"/>
@@ -4923,10 +4927,16 @@
       <c r="B122" s="4"/>
       <c r="C122" s="2"/>
     </row>
+    <row r="123" spans="1:3">
+      <c r="A123" s="2"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:C122"/>
-  <mergeCells count="1">
+  <autoFilter ref="A3:C1048576"/>
+  <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4937,16 +4947,15 @@
   <sheetPr>
     <tabColor rgb="FF7F7F7F"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28" customHeight="1">
+    <row r="1" spans="1:3" ht="28" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Настройки и справочники</t>
@@ -4954,9 +4963,8 @@
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:4" ht="22" customHeight="1">
+    </row>
+    <row r="2" spans="1:3" ht="22" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Категории</t>
@@ -4972,13 +4980,8 @@
           <t>Статусы</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Сотрудники</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Документы</t>
@@ -4994,13 +4997,8 @@
           <t>Новая</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Сотрудник 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Закупки</t>
@@ -5016,13 +5014,8 @@
           <t>В работе</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Сотрудник 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Встречи</t>
@@ -5038,13 +5031,8 @@
           <t>На паузе</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Сотрудник 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>IT</t>
@@ -5056,13 +5044,8 @@
           <t>Выполнено</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Сотрудник 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Администрирование</t>
@@ -5070,13 +5053,8 @@
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Сотрудник 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Прочее</t>
@@ -5084,12 +5062,11 @@
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D8"/>
+  <autoFilter ref="A2:C8"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand PTO task categories
Co-authored-by: DenisBerezovski1 <DenisBerezovski1@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/office_task_tracker.xlsx
+++ b/office_task_tracker.xlsx
@@ -11,9 +11,9 @@
     <sheet name="Настройки" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="task_categories">'Настройки'!$A$3:$A$8</definedName>
-    <definedName name="task_priorities">'Настройки'!$B$3:$B$5</definedName>
-    <definedName name="task_statuses">'Настройки'!$C$3:$C$6</definedName>
+    <definedName name="task_categories">'Настройки'!$A$3:INDEX('Настройки'!$A:$A,IFERROR(LOOKUP(2,1/(NOT(ISBLANK('Настройки'!$A$3:$A$1048576))),ROW('Настройки'!$A$3:$A$1048576)),3))</definedName>
+    <definedName name="task_priorities">'Настройки'!$B$3:INDEX('Настройки'!$B:$B,IFERROR(LOOKUP(2,1/(NOT(ISBLANK('Настройки'!$B$3:$B$1048576))),ROW('Настройки'!$B$3:$B$1048576)),3))</definedName>
+    <definedName name="task_statuses">'Настройки'!$C$3:INDEX('Настройки'!$C:$C,IFERROR(LOOKUP(2,1/(NOT(ISBLANK('Настройки'!$C$3:$C$1048576))),ROW('Настройки'!$C$3:$C$1048576)),3))</definedName>
     <definedName name="contact_names">'Контакты'!$A$4:INDEX('Контакты'!$A:$A,IFERROR(LOOKUP(2,1/(NOT(ISBLANK('Контакты'!$A$4:$A$1048576))),ROW('Контакты'!$A$4:$A$1048576)),4))</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -4947,7 +4947,7 @@
   <sheetPr>
     <tabColor rgb="FF7F7F7F"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -4984,7 +4984,7 @@
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Документы</t>
+          <t>Исполнительная документация</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -5001,7 +5001,7 @@
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Закупки</t>
+          <t>Акты скрытых работ</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -5018,7 +5018,7 @@
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Встречи</t>
+          <t>КС-2 / КС-3</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -5035,7 +5035,7 @@
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Сметы и расчеты</t>
         </is>
       </c>
       <c r="B6" s="4"/>
@@ -5048,7 +5048,7 @@
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Администрирование</t>
+          <t>Ведомости объемов работ</t>
         </is>
       </c>
       <c r="B7" s="4"/>
@@ -5057,14 +5057,122 @@
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Договоры и допсоглашения</t>
         </is>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Согласования</t>
+        </is>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Письма и деловая переписка</t>
+        </is>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Графики производства работ</t>
+        </is>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Поставки и материалы</t>
+        </is>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Проектная документация</t>
+        </is>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Рабочая документация</t>
+        </is>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Замечания и предписания</t>
+        </is>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Технические совещания</t>
+        </is>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Заявки и закупки</t>
+        </is>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Отчетность</t>
+        </is>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Архив и реестры</t>
+        </is>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Прочее</t>
+        </is>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:C8"/>
+  <autoFilter ref="A2:C20"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>

</xml_diff>